<commit_message>
escribo bien el reporte
</commit_message>
<xml_diff>
--- a/data/onedrive/alumnos_carrera.xlsx
+++ b/data/onedrive/alumnos_carrera.xlsx
@@ -1,15 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29523"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_200D2182D24D280F62355476585DCE3A875CE99D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EEDD8280-560B-47D3-B6F5-F2ACCEE28EE1}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_200D2182D24D280F62355476585DCE3A875CE99D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5BC0428-B0E9-48B7-B23F-F6AD62E43074}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$10532</definedName>
+  </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -86330,6 +86333,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:A10532" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>